<commit_message>
R2 - Issues fixed, missing list of tables and programs in README
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/econ0763/Downloads/JPE/JPE-Tincani-20230441/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA5860D-B1C4-C04E-9D24-35FBA01D3E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828DA77C-E48C-B043-AF11-16F87895348D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="402">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -1231,12 +1231,6 @@
   </si>
   <si>
     <t>yes</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>Values differ: Treatment col.2 0.264 vs 0.247, col.4 0.134 vs 0.152, col.6 0.022 vs 0.021; obs. 315 vs 316.</t>
   </si>
 </sst>
 </file>
@@ -2913,11 +2907,9 @@
         <v>267</v>
       </c>
       <c r="D98" t="s">
-        <v>402</v>
-      </c>
-      <c r="E98" s="4" t="s">
-        <v>403</v>
-      </c>
+        <v>401</v>
+      </c>
+      <c r="E98" s="4"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">

</xml_diff>